<commit_message>
new about and faq
</commit_message>
<xml_diff>
--- a/meta/faq.xlsx
+++ b/meta/faq.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\mig\Data Explorer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3F4879-6461-4CB7-AF50-60703D051300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068D94FC-BA80-4A37-B59A-0261ED0BEBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="faq" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="80">
   <si>
     <t>category</t>
   </si>
@@ -351,6 +351,18 @@
   </si>
   <si>
     <t>What is different in &lt;strong&gt; versions 3.1and 3.2&lt;strong&gt; ?</t>
+  </si>
+  <si>
+    <t>For the 66 countries listed here, estimates of the distribution of educational attainment (split) for post-secondary education were available: Bulgaria, Canada, Chile, China, China, Taiwan Province of China, Colombia, Croatia, Czechia, Denmark, Estonia, Finland, France, Georgia, State of Palestine, Germany, Greece, Argentina, China, Hong Kong SAR, Hungary, Iceland, Australia, Indonesia, Ireland, Israel, Italy, Austria, Jordan, Kenya, Republic of Korea, Latvia, Lithuania, Luxembourg, Maldives, Bahrain, Mexico, Montenegro, Mozambique, Netherlands, New Zealand, Belgium, Norway, Panama, Peru, Poland, Portugal, Puerto Rico, Romania, Saint Lucia, Bolivia (Plurinational State of), Saudi Arabia, Bosnia and Herzegovina, Slovakia, Viet Nam, Slovenia, South Africa, Botswana, Spain, Sweden, Switzerland, Syrian Arab Republic, Uganda, Egypt, United Kingdom, Belize, United States of America, and Uruguay.</t>
+  </si>
+  <si>
+    <t>For which countries are data available by eight levels of educational attainment?</t>
+  </si>
+  <si>
+    <t>How is the post-secondary category split into three educational levels?</t>
+  </si>
+  <si>
+    <t>The split is based on the distribution observed in the most recent year for which detailed data were available. This most recent distribution was then used to allocate the post‑secondary category into three sub‑levels—short post‑secondary, Bachelor’s, and Master’s+—for all future periods and scenarios. This approach ensures internal consistency across projections while preserving the relative composition of post‑secondary attainment.</t>
   </si>
 </sst>
 </file>
@@ -1235,15 +1247,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="107.28515625" customWidth="1"/>
-    <col min="3" max="3" width="255.5703125" customWidth="1"/>
+    <col min="2" max="2" width="107.26953125" customWidth="1"/>
+    <col min="3" max="3" width="255.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1254,7 +1266,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1265,7 +1277,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1276,7 +1288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1287,7 +1299,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1298,7 +1310,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1309,7 +1321,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1320,7 +1332,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1331,7 +1343,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1342,7 +1354,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1353,7 +1365,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1364,7 +1376,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1375,7 +1387,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1386,7 +1398,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1397,7 +1409,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1408,7 +1420,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="34.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="31" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -1419,7 +1431,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1430,7 +1442,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -1441,7 +1453,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -1452,7 +1464,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1463,7 +1475,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1474,7 +1486,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1485,7 +1497,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>26</v>
       </c>
@@ -1496,7 +1508,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1507,7 +1519,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -1518,7 +1530,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -1529,7 +1541,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1540,7 +1552,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -1551,7 +1563,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>53</v>
       </c>
@@ -1562,7 +1574,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>53</v>
       </c>
@@ -1573,7 +1585,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>53</v>
       </c>
@@ -1584,7 +1596,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="78" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="78.5" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -1595,7 +1607,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1606,7 +1618,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>26</v>
       </c>
@@ -1617,7 +1629,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>26</v>
       </c>
@@ -1628,7 +1640,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -1637,6 +1649,28 @@
       </c>
       <c r="C36" s="7" t="s">
         <v>73</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
+        <v>77</v>
+      </c>
+      <c r="C37" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>3</v>
+      </c>
+      <c r="B38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>